<commit_message>
UI update: default to all students filter, expand vertical panels to 620px, move excel upload to top header button
</commit_message>
<xml_diff>
--- a/data/master_bills.xlsx
+++ b/data/master_bills.xlsx
@@ -3988,13 +3988,27 @@
       </c>
       <c r="I62" t="inlineStr">
         <is>
-          <t>미납</t>
-        </is>
-      </c>
-      <c r="J62" t="inlineStr"/>
-      <c r="K62" t="inlineStr"/>
-      <c r="L62" t="inlineStr"/>
-      <c r="M62" t="inlineStr"/>
+          <t>수납</t>
+        </is>
+      </c>
+      <c r="J62" t="inlineStr">
+        <is>
+          <t>간편결제</t>
+        </is>
+      </c>
+      <c r="K62" t="inlineStr">
+        <is>
+          <t>네이버페이체크</t>
+        </is>
+      </c>
+      <c r="L62" t="inlineStr">
+        <is>
+          <t>2026-10-12 15:02:34</t>
+        </is>
+      </c>
+      <c r="M62" t="n">
+        <v>73864516</v>
+      </c>
       <c r="N62" t="inlineStr"/>
       <c r="O62" t="inlineStr"/>
       <c r="P62" t="inlineStr"/>

</xml_diff>

<commit_message>
Auto normalize new course names to standard canonical courses (e.g. 덕성여대, 인하대)
</commit_message>
<xml_diff>
--- a/data/master_bills.xlsx
+++ b/data/master_bills.xlsx
@@ -665,7 +665,7 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>미납</t>
+          <t>파기</t>
         </is>
       </c>
       <c r="K4" t="inlineStr"/>
@@ -675,8 +675,16 @@
       <c r="O4" t="inlineStr"/>
       <c r="P4" t="inlineStr"/>
       <c r="Q4" t="inlineStr"/>
-      <c r="R4" t="inlineStr"/>
-      <c r="S4" t="inlineStr"/>
+      <c r="R4" t="inlineStr">
+        <is>
+          <t>2026-10-20 17:32:08</t>
+        </is>
+      </c>
+      <c r="S4" t="inlineStr">
+        <is>
+          <t>전화번호 입력 오류</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -716,7 +724,7 @@
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>미납</t>
+          <t>파기</t>
         </is>
       </c>
       <c r="K5" t="inlineStr"/>
@@ -726,8 +734,16 @@
       <c r="O5" t="inlineStr"/>
       <c r="P5" t="inlineStr"/>
       <c r="Q5" t="inlineStr"/>
-      <c r="R5" t="inlineStr"/>
-      <c r="S5" t="inlineStr"/>
+      <c r="R5" t="inlineStr">
+        <is>
+          <t>2026-10-20 17:31:58</t>
+        </is>
+      </c>
+      <c r="S5" t="inlineStr">
+        <is>
+          <t>전화번호 입력 오류</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">

</xml_diff>